<commit_message>
Merged comms into Node file + autogen progress + circular buffer implementation
</commit_message>
<xml_diff>
--- a/Autogen/Example_Memory_Map.xlsx
+++ b/Autogen/Example_Memory_Map.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="35">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -44,13 +44,7 @@
     <t xml:space="preserve">Default</t>
   </si>
   <si>
-    <t xml:space="preserve">NVM Offset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OTP Offset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Custom Type</t>
+    <t xml:space="preserve">NVM Storage</t>
   </si>
   <si>
     <t xml:space="preserve">Description</t>
@@ -72,6 +66,9 @@
   </si>
   <si>
     <t xml:space="preserve">NODE_ID_MAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
   </si>
   <si>
     <t xml:space="preserve">Store NVM</t>
@@ -417,14 +414,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="27.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -455,285 +453,235 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="C3" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="H7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="H8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="H9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I9" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C9" type="list">
       <formula1>"RO,RW"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B9" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H9" type="list">
+      <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -752,14 +700,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="27.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -790,285 +739,235 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="C3" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="H7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="H8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="I9" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C9" type="list">
       <formula1>"RO,RW"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B9" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H9" type="list">
+      <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Small autogen updates - hub cpp re-added, better float handling.
</commit_message>
<xml_diff>
--- a/Autogen/Example_Memory_Map.xlsx
+++ b/Autogen/Example_Memory_Map.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Example1" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="42">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
-    <t xml:space="preserve">Node ID</t>
+    <t xml:space="preserve">WRITE UINT8</t>
   </si>
   <si>
     <t xml:space="preserve">uint8_t</t>
@@ -62,70 +62,91 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NODE_ID_MAX</t>
+    <t xml:space="preserve">1</t>
   </si>
   <si>
     <t xml:space="preserve">NO</t>
   </si>
   <si>
-    <t xml:space="preserve">Store NVM</t>
+    <t xml:space="preserve">WRITE INT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int8_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ UINT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ INT8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint16_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE INT16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int16_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ UINT16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ INT16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32</t>
   </si>
   <si>
     <t xml:space="preserve">uint32_t</t>
   </si>
   <si>
-    <t xml:space="preserve">Restore Factory NVM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store OTP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Watchdog Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory Map Gen Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">49856</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory Map Gen Time</t>
+    <t xml:space="preserve">WRITE INT32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int32_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ UINT32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ INT32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE FLOAT</t>
   </si>
   <si>
     <t xml:space="preserve">float</t>
   </si>
   <si>
-    <t xml:space="preserve">4.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory Map Checksum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">int8_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint16_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64563</t>
-  </si>
-  <si>
-    <t xml:space="preserve">int32_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-655346</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0001</t>
+    <t xml:space="preserve">READ FLOAT</t>
   </si>
 </sst>
 </file>
@@ -214,7 +235,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -229,6 +250,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -414,14 +439,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.49"/>
   </cols>
   <sheetData>
@@ -468,43 +493,43 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I3" s="3"/>
     </row>
@@ -513,10 +538,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>12</v>
@@ -528,23 +553,23 @@
         <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
@@ -555,19 +580,19 @@
         <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>11</v>
@@ -582,22 +607,22 @@
         <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>12</v>
@@ -609,22 +634,22 @@
         <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>12</v>
@@ -636,22 +661,22 @@
         <v>12</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>12</v>
@@ -663,24 +688,186 @@
         <v>12</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C15" type="list">
       <formula1>"RO,RW"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B15" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H15" type="list">
       <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -700,14 +887,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.49"/>
   </cols>
   <sheetData>
@@ -754,43 +941,43 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I3" s="3"/>
     </row>
@@ -799,10 +986,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>12</v>
@@ -814,23 +1001,23 @@
         <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="D5" s="3" t="s">
         <v>12</v>
       </c>
@@ -841,19 +1028,19 @@
         <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>11</v>
@@ -868,22 +1055,22 @@
         <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>12</v>
@@ -895,22 +1082,22 @@
         <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>12</v>
@@ -922,22 +1109,22 @@
         <v>12</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>12</v>
@@ -949,24 +1136,180 @@
         <v>12</v>
       </c>
       <c r="G9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C15" type="list">
       <formula1>"RO,RW"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B15" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H9" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H15" type="list">
       <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Updates to universal memory map functionality in progress Node side
</commit_message>
<xml_diff>
--- a/Autogen/Example_Memory_Map.xlsx
+++ b/Autogen/Example_Memory_Map.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Example1" sheetId="1" state="visible" r:id="rId3"/>
@@ -65,7 +65,7 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">NO</t>
+    <t xml:space="preserve">false</t>
   </si>
   <si>
     <t xml:space="preserve">WRITE INT8</t>
@@ -868,7 +868,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H15" type="list">
-      <formula1>"NO,YES"</formula1>
+      <formula1>"true,false"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1310,7 +1310,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H15" type="list">
-      <formula1>"NO,YES"</formula1>
+      <formula1>"true,false"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>